<commit_message>
navbar responsive fixed + roles modifications
</commit_message>
<xml_diff>
--- a/test1.xlsx
+++ b/test1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28014"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\marmina\api\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\marmina\api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98722DCD-F475-4B50-B027-3B8201A395F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F3247C6-95AF-4EF3-8ECE-A635A6A1400F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1391,30 +1391,63 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="13" fillId="6" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1427,35 +1460,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1463,10 +1467,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="13" fillId="6" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2099,13 +2099,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="76" t="s">
+      <c r="B1" s="93" t="s">
         <v>65</v>
       </c>
-      <c r="C1" s="80" t="s">
+      <c r="C1" s="68" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="66"/>
@@ -2124,17 +2124,17 @@
       <c r="Q1" s="66"/>
       <c r="R1" s="66"/>
       <c r="S1" s="66"/>
-      <c r="T1" s="79"/>
+      <c r="T1" s="67"/>
     </row>
     <row r="2" spans="1:20" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="70"/>
-      <c r="B2" s="77"/>
+      <c r="A2" s="72"/>
+      <c r="B2" s="94"/>
       <c r="C2" s="65" t="s">
         <v>3</v>
       </c>
       <c r="D2" s="66"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="68"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="91"/>
       <c r="G2" s="65" t="s">
         <v>4</v>
       </c>
@@ -2144,81 +2144,81 @@
       <c r="K2" s="66"/>
       <c r="L2" s="66"/>
       <c r="M2" s="66"/>
-      <c r="N2" s="79"/>
+      <c r="N2" s="67"/>
       <c r="O2" s="65" t="s">
         <v>5</v>
       </c>
       <c r="P2" s="66"/>
       <c r="Q2" s="66"/>
-      <c r="R2" s="79"/>
-      <c r="S2" s="69" t="s">
+      <c r="R2" s="67"/>
+      <c r="S2" s="71" t="s">
         <v>6</v>
       </c>
-      <c r="T2" s="82" t="s">
+      <c r="T2" s="73" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="70"/>
-      <c r="B3" s="77"/>
-      <c r="C3" s="72" t="s">
+      <c r="A3" s="72"/>
+      <c r="B3" s="94"/>
+      <c r="C3" s="84" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="74" t="s">
+      <c r="D3" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="63" t="s">
+      <c r="E3" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="63" t="s">
+      <c r="F3" s="82" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="88" t="s">
+      <c r="G3" s="80" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="85" t="s">
+      <c r="H3" s="76" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="85" t="s">
+      <c r="I3" s="76" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="93" t="s">
+      <c r="J3" s="88" t="s">
         <v>15</v>
       </c>
-      <c r="K3" s="91" t="s">
+      <c r="K3" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="L3" s="92"/>
-      <c r="M3" s="92"/>
-      <c r="N3" s="81" t="s">
+      <c r="L3" s="87"/>
+      <c r="M3" s="87"/>
+      <c r="N3" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="O3" s="72" t="s">
+      <c r="O3" s="84" t="s">
         <v>18</v>
       </c>
-      <c r="P3" s="85" t="s">
+      <c r="P3" s="76" t="s">
         <v>19</v>
       </c>
-      <c r="Q3" s="74" t="s">
+      <c r="Q3" s="78" t="s">
         <v>20</v>
       </c>
-      <c r="R3" s="81" t="s">
+      <c r="R3" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="S3" s="70"/>
-      <c r="T3" s="83"/>
+      <c r="S3" s="72"/>
+      <c r="T3" s="74"/>
     </row>
     <row r="4" spans="1:20" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="71"/>
-      <c r="B4" s="78"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="90"/>
-      <c r="G4" s="89"/>
-      <c r="H4" s="86"/>
-      <c r="I4" s="86"/>
-      <c r="J4" s="86"/>
+      <c r="A4" s="70"/>
+      <c r="B4" s="95"/>
+      <c r="C4" s="85"/>
+      <c r="D4" s="92"/>
+      <c r="E4" s="89"/>
+      <c r="F4" s="83"/>
+      <c r="G4" s="81"/>
+      <c r="H4" s="77"/>
+      <c r="I4" s="77"/>
+      <c r="J4" s="77"/>
       <c r="K4" s="1" t="s">
         <v>22</v>
       </c>
@@ -2228,13 +2228,13 @@
       <c r="M4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N4" s="71"/>
-      <c r="O4" s="73"/>
-      <c r="P4" s="86"/>
-      <c r="Q4" s="87"/>
-      <c r="R4" s="71"/>
-      <c r="S4" s="71"/>
-      <c r="T4" s="84"/>
+      <c r="N4" s="70"/>
+      <c r="O4" s="85"/>
+      <c r="P4" s="77"/>
+      <c r="Q4" s="79"/>
+      <c r="R4" s="70"/>
+      <c r="S4" s="70"/>
+      <c r="T4" s="75"/>
     </row>
     <row r="5" spans="1:20" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
@@ -4176,10 +4176,10 @@
       </c>
     </row>
     <row r="34" spans="1:20" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="98" t="s">
+      <c r="A34" s="64" t="s">
         <v>96</v>
       </c>
-      <c r="B34" s="97" t="s">
+      <c r="B34" s="63" t="s">
         <v>95</v>
       </c>
       <c r="C34" s="25">
@@ -8684,6 +8684,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="A1:A4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="B1:B4"/>
     <mergeCell ref="G2:N2"/>
     <mergeCell ref="O2:R2"/>
     <mergeCell ref="C1:T1"/>
@@ -8700,12 +8706,6 @@
     <mergeCell ref="N3:N4"/>
     <mergeCell ref="I3:I4"/>
     <mergeCell ref="J3:J4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="C2:F2"/>
-    <mergeCell ref="A1:A4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="B1:B4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
@@ -8730,13 +8730,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="96" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="96"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="98"/>
     </row>
     <row r="2" spans="1:12" s="40" customFormat="1" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="39" t="s">

</xml_diff>